<commit_message>
RBM Classification report classifies by the directive's bands by term (workbook 4 finding F3 closed)
The report, the provision comparison and the arrears ageing used one ladder (90/180/365 days, 1 percent on pass and special mention). They now classify by the directive's bands by term of facility (30/90/180/360 short-term, 30/180/360/720 medium and long) at the directive's rates (0/5/20/50/100), from one SQL rule mirroring RbmReturnService::classify; the arrears ageing shows the class beside each day band since the band alone no longer decides it. A test proves the report and the return agree at every band edge on both terms.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/RBM_DFI_Directive_2018_Compliance_Audit.xlsx
+++ b/docs/compliance/RBM_DFI_Directive_2018_Compliance_Audit.xlsx
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E8" s="22" t="inlineStr">
         <is>
-          <t>The RBM Classification report classifies each loan from the days past due the build counts from the oldest overdue instalment, with the bucket ageing beside it; the IFRS 9 stage is mapped to the RBM class in the IFRS 9 vs RBM report.</t>
+          <t>The RBM Classification report classifies each loan from the days past due the build counts from the oldest overdue instalment, under the directive's bands by term of facility (the same bands as the RBM Return, proven to agree at every band edge); the arrears ageing shows the class beside each day band; the IFRS 9 stage is mapped to the RBM class in the IFRS 9 vs RBM report.</t>
         </is>
       </c>
       <c r="F8" s="22" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="K8" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\StagingServiceTest</t>
+          <t>Tests\Feature\Rbm\RbmReturnServiceTest::test_the_rbm_classification_report_agrees_with_the_return_on_every_loan</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>The RBM Classification report applies the day bands; the loan book's buckets end at 271 to 360 days and the build counts days from the overdue date without a ceiling, so the doubtful and loss bands are classified from the day count; the qualitative 'recovery not expected' flag is the write-off policy MAIIC has not stated.</t>
+          <t>The RBM Classification report and the RBM Return apply the doubtful and loss bands by term (181/361 days short-term, 361/721 otherwise); the loan book's buckets end at 271 to 360 days and the build counts days from the overdue date without a ceiling, so the bands are classified from the day count; the qualitative 'recovery not expected' flag is the write-off policy MAIIC has not stated.</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr"/>
@@ -1344,7 +1344,7 @@
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\StagingServiceTest</t>
+          <t>Tests\Feature\Rbm\RbmReturnServiceTest</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1779,22 @@
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>The RBM Classification report's day bands differ from the directive's</t>
+          <t>The RBM Classification report's day bands differed from the directive's</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>The older RBM Classification report classifies every facility on one ladder (90, 180, 365 days); the directive classifies by term (90/180/360 for short-term, 180/360/720 for medium and long). The provisional return applies the directive's bands.</t>
+          <t>The older RBM Classification report classified every facility on one ladder (90, 180, 365 days) with 1 percent on pass and special mention; the directive classifies by term (90/180/360 for short-term, 180/360/720 for medium and long) with 0 and 5 percent. Resolved 9 October 2026: the report, the provision comparison and the arrears ageing now classify by the directive's bands by term and rates, from the same rule as the return; a test proves the two agree at every band edge on both terms.</t>
         </is>
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>The two screens can show different classes for the same medium-term facility.</t>
+          <t>None remaining: the two screens show one class for every facility.</t>
         </is>
       </c>
       <c r="F7" s="22" t="inlineStr">
         <is>
-          <t>Align the RBM Classification report to the directive's bands by term (or retire it in favour of the return).</t>
+          <t>Done.</t>
         </is>
       </c>
       <c r="G7" s="22" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-08 21:50:42 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
+          <t>Generated 2026-10-08 22:00:02 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RBM bands corrected to the Gazette; compliance PDF footer names MAIIC
The system audit of 9 October 2026 found the RBM classification bands built on 8 October (30/90/180/360 short-term, 30/180/360/720 medium and long) came from a note carried between sessions, not from the directive. Section 10 of the Gazette (docs/regulatory, pages 683 and 685) has short-term 30/90/180/365 and medium and long term 90/180/365/746: a medium-term facility 31 to 90 days overdue is standard at 0 percent, not special mention at 5. RbmReturnService, the RBM Classification report, the provision comparison and the arrears ageing now carry the Gazette's bands; the test asserts every boundary on both terms (it had asserted the wrong ones). Workbook 4 finding F3 records both corrections.

tools/compliance/md_to_pdf.py printed another client's name in the footer of every compliance PDF; the five workbooks are regenerated with "MAIIC IFRS 9".

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/RBM_DFI_Directive_2018_Compliance_Audit.xlsx
+++ b/docs/compliance/RBM_DFI_Directive_2018_Compliance_Audit.xlsx
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C10" s="22" t="inlineStr">
         <is>
-          <t>Doubtful from 181 (short-term) or 361 days (medium and long term); loss from 361 or 721 days, or where recovery is not expected.</t>
+          <t>Doubtful from 181 (short-term) or 366 days (medium and long term); loss beyond 365 or 746 days, or where recovery is not expected.</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>The RBM Classification report and the RBM Return apply the doubtful and loss bands by term (181/361 days short-term, 361/721 otherwise); the loan book's buckets end at 271 to 360 days and the build counts days from the overdue date without a ceiling, so the bands are classified from the day count; the qualitative 'recovery not expected' flag is the write-off policy MAIIC has not stated.</t>
+          <t>The RBM Classification report and the RBM Return apply the doubtful and loss bands by term from section 10 of the Gazette (181/366 days short-term, 366/747 otherwise); the loan book's buckets end at 271 to 360 days and the build counts days from the overdue date without a ceiling, so the bands are classified from the day count; the qualitative 'recovery not expected' flag is the write-off policy MAIIC has not stated.</t>
         </is>
       </c>
       <c r="F10" s="22" t="inlineStr"/>
@@ -1784,12 +1784,12 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>The older RBM Classification report classified every facility on one ladder (90, 180, 365 days) with 1 percent on pass and special mention; the directive classifies by term (90/180/360 for short-term, 180/360/720 for medium and long) with 0 and 5 percent. Resolved 9 October 2026: the report, the provision comparison and the arrears ageing now classify by the directive's bands by term and rates, from the same rule as the return; a test proves the two agree at every band edge on both terms.</t>
+          <t>The older RBM Classification report classified every facility on one ladder (90, 180, 365 days) with 1 percent on pass and special mention. Resolved in two steps: on 9 October 2026 the report, the provision comparison and the arrears ageing were put on one rule with the RBM Return; the system audit of the same day then found that rule itself carried wrong medium- and long-term bands (30/180/360/720, from a note carried between sessions) and both were corrected to the Gazette's section 10: short-term 30/90/180/365, medium and long 90/180/365/746, with a test at every boundary on both terms.</t>
         </is>
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>None remaining: the two screens show one class for every facility.</t>
+          <t>None remaining: both screens classify by the Gazette's bands.</t>
         </is>
       </c>
       <c r="F7" s="22" t="inlineStr">
@@ -1859,7 +1859,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-08 22:00:02 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
+          <t>Generated 2026-10-09 00:03:49 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
         </is>
       </c>
     </row>

</xml_diff>